<commit_message>
docs(tutorials): FEM-3's geogrid layers are 5 m long; the geogrid wall re-locks at 1.246
Three 3 m layers in a 6 m reinforced zone looked wrong; at 5 m they reach most of the way through it. The model is rebuilt through the builder, the sketch and the reinforcement editor screenshot follow, the mesh grows to 2,139 nodes and 90 joint elements, and every Part 2 panel is redrawn from the new solve in both field states. The slip comparison, the 1D Details reading and the strain reading hold at the same numbers.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XjjT2aBxw8gY7EFdpoUcpj
</commit_message>
<xml_diff>
--- a/docs/tutorials/files/xslope_block_wall_grid.xlsx
+++ b/docs/tutorials/files/xslope_block_wall_grid.xlsx
@@ -3764,7 +3764,7 @@
         <v>0.6</v>
       </c>
       <c r="E3" s="3">
-        <v>12.2</v>
+        <v>14.2</v>
       </c>
       <c r="F3" s="3">
         <v>0.6</v>
@@ -3851,7 +3851,7 @@
         <v>1.8</v>
       </c>
       <c r="E4" s="3">
-        <v>12.2</v>
+        <v>14.2</v>
       </c>
       <c r="F4" s="3">
         <v>1.8</v>
@@ -3932,7 +3932,7 @@
         <v>3.0</v>
       </c>
       <c r="E5" s="3">
-        <v>12.2</v>
+        <v>14.2</v>
       </c>
       <c r="F5" s="3">
         <v>3.0</v>

</xml_diff>